<commit_message>
AFK backlog clear: CR cascade, Wave1 residual, research, Swing verify
Phase 0: MASTER-LEDGER + geometry refresh (story-hold 0; mesh deferred).

Phase 3A: DiDi Costa Rica cascade — grounded 7→9, floor +$1.57M, sheet uploaded.

Phase 1: Wave1 BP research ledger (0 false T2 seals); mint Elbląg→Krynica after
schedule proof; 13 residual routes remain endpoint-blocked honestly.

Phase 3B–D/4: AR/VE/caribbean research holds retained with receipts; Constance
diagnosed (captive fraction); saudi-pif/RSG audited + sheets rebuilt.

Phase 5: Swing deck verified release-ready (loss mid-case, six OPEX, 1PxUt links,
SOM floor $10,453,754).

No invented rates/coords/demand. Null beats wrong.
</commit_message>
<xml_diff>
--- a/finance/_refresh_red-sea-global.xlsx
+++ b/finance/_refresh_red-sea-global.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Country opex" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Corridor economics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Market sizing" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Economics holds" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Corridor economics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Market sizing" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="pax_cap">'Assumptions'!$B$5</definedName>
@@ -148,12 +149,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5A88"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="002E5A88"/>
       </patternFill>
     </fill>
     <fill>
@@ -188,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -211,9 +212,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,8 +245,8 @@
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -251,7 +255,7 @@
     <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -261,6 +265,7 @@
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -304,7 +309,7 @@
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -326,10 +331,10 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -337,6 +342,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -707,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B36"/>
+  <dimension ref="B2:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -925,6 +933,13 @@
       <c r="B36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Every fare &amp; demand figure carries a Source tier (T1 official → T5 modeled) + Confidence (high/med/low). Null beats a wrong number: no published pool → blank, not a guess.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Economics holds: 0 corridor(s) are explicitly excluded; see the Economics holds tab. Missing country costs never borrow Singapore or another market.</t>
         </is>
       </c>
     </row>
@@ -951,841 +966,841 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Assumptions — single source of truth (the engine references these named cells)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Vessel — N30 Pioneer II  (L1 global, commercial now)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Conf.</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Passenger capacity</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>pax</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Navier model: up to 8 pax where local rules allow (Jaideep set base case to 8, 2026-06-06)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>nm</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Navier locked spec (KB)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Cruise speed</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>kt</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>Navier locked spec (cruise)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>CAPEX (per vessel; US/EU base — ROW=$600K, see Country opex tab col G)</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <v>900000</v>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>Navier price (LYFT ref model, ex tax/fees)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Battery</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="13" t="n">
         <v>114</v>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>kWh</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Navier data (LYFT ref model)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Annual maintenance</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <v>10000</v>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>USD/yr</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Navier data (LYFT ref model)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Depreciation life</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>yr</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Marine-vessel market best practice (Jaideep locked 2026-06-07): commercial passenger vessels straight-line over ~20-25yr useful life; corroborated by Sampriti founder Jan-2024 operating model (20yr). Was placeholder 10yr.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Diesel comparable economy</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>nm/gal</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>Navier + open web (LYFT ref model)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Operating defaults  (L1 global; overridable per market)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Conf.</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Service window</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>hr/day</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Modeled single-asset commercial service window (one extended crew day, water-taxi norm). Conservative vs 24h.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Turnaround / charge per leg</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>Navier fast-charge (LYFT ref ~20-30min)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Boarding / scheduling dwell per leg</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Premium board/deboard + scheduling slack added to each cycle (Jaideep 2026-06-19).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Max revenue sailings/day (cap)</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>legs/day</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Cap on revenue sailings/day — 15 across thin/mid/full scenarios (Jaideep 2026-06-21).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Crew FTE factor (x captain wage)</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n">
+      <c r="B20" s="17" t="n">
         <v>1.8</v>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>A captain can't run 7 days/wk; 1.8 FTE covers relief/leave/second-shift year-round (Jaideep 2026-06-19). Scales off localized captain wage.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Mechanical uptime</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B21" s="18" t="n">
         <v>0.75</v>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Blade luxury aviation ~75-80% reliability uptime</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Navier capture rate</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr"/>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr"/>
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>Navier wins ~10% of a CONTESTED corridor demand pool (locked). Captive sole-operator transfer legs (captive:true / luxury_charter / hospitality archetypes) carry the captive rate instead — see per-row Capture %.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Captive capture rate (A′ corridors)</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr"/>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>Sole-operator water-access-only transfer legs (captive:true or luxury_charter/hospitality archetype): Navier IS the transfer fleet — capture ~90%. Applied per-row in the Capture % column.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Discount factor (vs comparable fare)</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>Market parity — better product, not cheaper (locked).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Diesel CO₂ per gallon</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B25" s="17" t="n">
         <v>10.21</v>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>kg/gal</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>US EPA: 10.21 kg CO2 per gallon marine/diesel</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>OPEX defaults  (global fallbacks — localized energy, crew, berth admin on Country opex tab)</t>
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>OPEX defaults  (global vessel assumptions — country costs use exact-key rows only)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Conf.</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Vessel insurance — H&amp;M + P&amp;I (% of CAPEX/yr)</t>
         </is>
       </c>
-      <c r="B29" s="17" t="n">
+      <c r="B29" s="18" t="n">
         <v>0.025</v>
       </c>
-      <c r="C29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>Commercial vessel H&amp;M + P&amp;I ~2.5%/yr of regional CAPEX. Separate from berth/port admin in Country opex (Jaideep 2026-06-19).. Multiplied by regional CAPEX (Country opex col G). Not included in berth/port admin.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Fast-charge berth &amp; demand charges (global default)</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B30" s="16" t="n">
         <v>18000</v>
       </c>
-      <c r="C30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>USD/yr</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>Dedicated fast-charge berth slot + utility demand charges. Excludes per-kWh propulsion energy and berth/port admin (Jaideep 2026-06-19). L3-overridable per market.. Dedicated charge berth + utility demand charges. Excludes per-kWh propulsion energy and berth/port admin. L3-overridable per market.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Utilization scenarios  (load factor + revenue-leg factor)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Load factor</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>Rev-leg factor</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr"/>
-      <c r="E33" s="10" t="inlineStr"/>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr"/>
+      <c r="E33" s="11" t="inlineStr"/>
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>THIN</t>
         </is>
       </c>
-      <c r="B34" s="19" t="n">
+      <c r="B34" s="20" t="n">
         <v>0.45</v>
       </c>
-      <c r="C34" s="19" t="n">
+      <c r="C34" s="20" t="n">
         <v>0.55</v>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>thin/one-way/seasonal corridor — conservative floor</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="B35" s="19" t="n">
+      <c r="B35" s="20" t="n">
         <v>0.55</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C35" s="20" t="n">
         <v>0.65</v>
       </c>
-      <c r="F35" s="14" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
         <is>
           <t>HEADLINE — realistic busy two-way corridor</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>FULL</t>
         </is>
       </c>
-      <c r="B36" s="19" t="n">
+      <c r="B36" s="20" t="n">
         <v>0.7</v>
       </c>
-      <c r="C36" s="19" t="n">
+      <c r="C36" s="20" t="n">
         <v>0.75</v>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F36" s="15" t="inlineStr">
         <is>
           <t>mature/dense corridor — optimistic ceiling</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>SCENARIO (toggle me)</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="C38" s="22" t="inlineStr">
+      <c r="C38" s="23" t="inlineStr">
         <is>
           <t>← set THIN / MID / FULL</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Selected load factor</t>
         </is>
       </c>
-      <c r="B39" s="23">
+      <c r="B39" s="24">
         <f>VLOOKUP(scenario,'Assumptions'!$A$34:$C$36,2,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Selected rev-leg factor</t>
         </is>
       </c>
-      <c r="B40" s="23">
+      <c r="B40" s="24">
         <f>VLOOKUP(scenario,'Assumptions'!$A$34:$C$36,3,FALSE)</f>
         <v/>
       </c>
@@ -1827,79 +1842,79 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Country opex — localized inputs (crew, energy, berth admin, CAPEX)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>Captain $/yr</t>
         </is>
       </c>
-      <c r="C3" s="24" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>Energy $/kWh</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" s="25" t="inlineStr">
         <is>
           <t>Grid CO₂ kg/kWh</t>
         </is>
       </c>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>Berth &amp; port admin $/yr</t>
         </is>
       </c>
-      <c r="F3" s="24" t="inlineStr">
+      <c r="F3" s="25" t="inlineStr">
         <is>
           <t>Cost index</t>
         </is>
       </c>
-      <c r="G3" s="24" t="inlineStr">
+      <c r="G3" s="25" t="inlineStr">
         <is>
           <t>CAPEX $/vessel</t>
         </is>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="25" t="inlineStr">
         <is>
           <t>Source notes (crew | energy | berth admin)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="B4" s="27" t="n">
         <v>42000</v>
       </c>
-      <c r="C4" s="27" t="n">
+      <c r="C4" s="28" t="n">
         <v>0.074</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="20" t="n">
         <v>0.57</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="20" t="n">
         <v>0.68</v>
       </c>
-      <c r="G4" s="26" t="n">
+      <c r="G4" s="27" t="n">
         <v>600000</v>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>GCC expat marine crew. Job ads (Instagram/Facebook 2026): yacht/boat captain SAR 7,000-10,000/mo (~$1,870-2,670/mo); ERI SalaryExpert boat captain avg SAR 203,728/yr (~$54k, high-side single qualified). Blended 1 commercial tourism-boat captain (~SAR 8,500/mo) + deckhand (~SAR 3,500/mo) fully-loaded (housing/food/visa typically provided) ~= SAR 157k = ~$42k/vessel/yr @3.75. High-income GCC; just below Singapore $48k. | HEAVILY SUBSIDIZED. SEC/SERA commercial tariff: SAR 0.22/kWh up to 6,000 kWh/mo, SAR 0.32 above (clenergize/SEC 2025). GlobalPetrolPrices business SAR 0.277 = $0.074 (Sep 2025). Anchored $0.074. Floor (low-band) ~$0.059, ceiling (high-band SAR 0.32) ~$0.085. @SAR 3.75 (pegged). | Modeled berth+insurance+admin/vessel/yr. New premium Red Sea Global / NEOM marinas (Shura, Sindalah 86-berth) are high-cost GCC marine ops; above Taiwan $14k, below Singapore $20k. Tagged low. | CAPEX LB-243 US/EU=$900K else $600K</t>
         </is>
@@ -1914,6 +1929,72 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="86" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Economics holds — excluded before model and sheet calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>Corridor</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>Route ID</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="inlineStr">
+        <is>
+          <t>Country label</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="inlineStr">
+        <is>
+          <t>Hold reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>None — all in-scope corridors have complete exact-key country references.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1976,1813 +2057,1813 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Navier × Red-Sea-Global — Corridor economics (one boat, one year; MID = headline)</t>
         </is>
       </c>
-      <c r="N1" s="28" t="inlineStr">
+      <c r="N1" s="30" t="inlineStr">
         <is>
           <t>SCENARIO:</t>
         </is>
       </c>
-      <c r="O1" s="21">
+      <c r="O1" s="22">
         <f>scenario</f>
         <v/>
       </c>
-      <c r="P1" s="22" t="inlineStr">
+      <c r="P1" s="23" t="inlineStr">
         <is>
           <t>(set on Assumptions tab)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C3" s="24" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>Corridor</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" s="25" t="inlineStr">
         <is>
           <t>Distance</t>
         </is>
       </c>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>Premium fare $/pax</t>
         </is>
       </c>
-      <c r="F3" s="24" t="inlineStr">
+      <c r="F3" s="25" t="inlineStr">
         <is>
           <t>Fare tier</t>
         </is>
       </c>
-      <c r="G3" s="24" t="inlineStr">
+      <c r="G3" s="25" t="inlineStr">
         <is>
           <t>Fare conf.</t>
         </is>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="25" t="inlineStr">
         <is>
           <t>Weather factor</t>
         </is>
       </c>
-      <c r="I3" s="24" t="inlineStr">
+      <c r="I3" s="25" t="inlineStr">
         <is>
           <t>One-way min</t>
         </is>
       </c>
-      <c r="J3" s="24" t="inlineStr">
+      <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Cycle min</t>
         </is>
       </c>
-      <c r="K3" s="24" t="inlineStr">
+      <c r="K3" s="25" t="inlineStr">
         <is>
           <t>Trips/day</t>
         </is>
       </c>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="25" t="inlineStr">
         <is>
           <t>Op days/yr</t>
         </is>
       </c>
-      <c r="M3" s="24" t="inlineStr">
+      <c r="M3" s="25" t="inlineStr">
         <is>
           <t>Mech uptime</t>
         </is>
       </c>
-      <c r="N3" s="24" t="inlineStr">
+      <c r="N3" s="25" t="inlineStr">
         <is>
           <t>Rev-leg %</t>
         </is>
       </c>
-      <c r="O3" s="24" t="inlineStr">
+      <c r="O3" s="25" t="inlineStr">
         <is>
           <t>Trips/yr</t>
         </is>
       </c>
-      <c r="P3" s="24" t="inlineStr">
+      <c r="P3" s="25" t="inlineStr">
         <is>
           <t>Load factor</t>
         </is>
       </c>
-      <c r="Q3" s="24" t="inlineStr">
+      <c r="Q3" s="25" t="inlineStr">
         <is>
           <t>Pax/trip</t>
         </is>
       </c>
-      <c r="R3" s="24" t="inlineStr">
+      <c r="R3" s="25" t="inlineStr">
         <is>
           <t>Pax/yr</t>
         </is>
       </c>
-      <c r="S3" s="24" t="inlineStr">
+      <c r="S3" s="25" t="inlineStr">
         <is>
           <t>Navier fare $</t>
         </is>
       </c>
-      <c r="T3" s="24" t="inlineStr">
+      <c r="T3" s="25" t="inlineStr">
         <is>
           <t>Revenue/yr</t>
         </is>
       </c>
-      <c r="U3" s="24" t="inlineStr">
+      <c r="U3" s="25" t="inlineStr">
         <is>
           <t>Energy/yr</t>
         </is>
       </c>
-      <c r="V3" s="24" t="inlineStr">
+      <c r="V3" s="25" t="inlineStr">
         <is>
           <t>Crew/yr</t>
         </is>
       </c>
-      <c r="W3" s="24" t="inlineStr">
+      <c r="W3" s="25" t="inlineStr">
         <is>
           <t>Berth &amp; port admin/yr</t>
         </is>
       </c>
-      <c r="X3" s="24" t="inlineStr">
+      <c r="X3" s="25" t="inlineStr">
         <is>
           <t>Maint/yr</t>
         </is>
       </c>
-      <c r="Y3" s="24" t="inlineStr">
+      <c r="Y3" s="25" t="inlineStr">
         <is>
           <t>Vessel insurance/yr</t>
         </is>
       </c>
-      <c r="Z3" s="24" t="inlineStr">
+      <c r="Z3" s="25" t="inlineStr">
         <is>
           <t>Fast-charge berth/yr</t>
         </is>
       </c>
-      <c r="AA3" s="24" t="inlineStr">
+      <c r="AA3" s="25" t="inlineStr">
         <is>
           <t>OPEX/yr</t>
         </is>
       </c>
-      <c r="AB3" s="24" t="inlineStr">
+      <c r="AB3" s="25" t="inlineStr">
         <is>
           <t>Deprec/yr</t>
         </is>
       </c>
-      <c r="AC3" s="24" t="inlineStr">
+      <c r="AC3" s="25" t="inlineStr">
         <is>
           <t>EBITDA/yr</t>
         </is>
       </c>
-      <c r="AD3" s="24" t="inlineStr">
+      <c r="AD3" s="25" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="AE3" s="24" t="inlineStr">
+      <c r="AE3" s="25" t="inlineStr">
         <is>
           <t>Payback yr (sel)</t>
         </is>
       </c>
-      <c r="AF3" s="24" t="inlineStr">
+      <c r="AF3" s="25" t="inlineStr">
         <is>
           <t>CO₂ saved t/yr</t>
         </is>
       </c>
-      <c r="AG3" s="24" t="inlineStr">
+      <c r="AG3" s="25" t="inlineStr">
         <is>
           <t>Demand pool 1-way/yr</t>
         </is>
       </c>
-      <c r="AH3" s="24" t="inlineStr">
+      <c r="AH3" s="25" t="inlineStr">
         <is>
           <t>Demand tier</t>
         </is>
       </c>
-      <c r="AI3" s="24" t="inlineStr">
+      <c r="AI3" s="25" t="inlineStr">
         <is>
           <t>Demand conf.</t>
         </is>
       </c>
-      <c r="AJ3" s="24" t="inlineStr">
+      <c r="AJ3" s="25" t="inlineStr">
         <is>
           <t>Capture %</t>
         </is>
       </c>
-      <c r="AK3" s="24" t="inlineStr">
+      <c r="AK3" s="25" t="inlineStr">
         <is>
           <t>Navier rides/yr</t>
         </is>
       </c>
-      <c r="AL3" s="24" t="inlineStr">
+      <c r="AL3" s="25" t="inlineStr">
         <is>
           <t>Vessels @capture</t>
         </is>
       </c>
-      <c r="AM3" s="24" t="inlineStr">
+      <c r="AM3" s="25" t="inlineStr">
         <is>
           <t>Market rev/yr</t>
         </is>
       </c>
-      <c r="AN3" s="24" t="inlineStr">
+      <c r="AN3" s="25" t="inlineStr">
         <is>
           <t>Vessels raw (unfloored)</t>
         </is>
       </c>
-      <c r="AO3" s="24" t="inlineStr">
+      <c r="AO3" s="25" t="inlineStr">
         <is>
           <t>Market rev/yr raw</t>
         </is>
       </c>
-      <c r="AP3" s="24" t="inlineStr">
+      <c r="AP3" s="25" t="inlineStr">
         <is>
           <t>Subset of (excl. from market fleet)</t>
         </is>
       </c>
-      <c r="AQ3" s="24" t="inlineStr">
+      <c r="AQ3" s="25" t="inlineStr">
         <is>
           <t>Floor bucket (aggregate status)</t>
         </is>
       </c>
-      <c r="AR3" s="24" t="inlineStr">
+      <c r="AR3" s="25" t="inlineStr">
         <is>
           <t>Forward SAM (2030-dated; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="AS3" s="24" t="inlineStr">
+      <c r="AS3" s="25" t="inlineStr">
         <is>
           <t>Upside tier (LB-99; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="AT3" s="24" t="inlineStr">
+      <c r="AT3" s="25" t="inlineStr">
         <is>
           <t>Fleet ceiling (captive villas/25)</t>
         </is>
       </c>
-      <c r="AU3" s="24" t="inlineStr">
+      <c r="AU3" s="25" t="inlineStr">
         <is>
           <t>Payback THIN</t>
         </is>
       </c>
-      <c r="AV3" s="24" t="inlineStr">
+      <c r="AV3" s="25" t="inlineStr">
         <is>
           <t>Payback MID</t>
         </is>
       </c>
-      <c r="AW3" s="24" t="inlineStr">
+      <c r="AW3" s="25" t="inlineStr">
         <is>
           <t>Payback FULL</t>
         </is>
       </c>
-      <c r="AX3" s="24" t="inlineStr">
+      <c r="AX3" s="25" t="inlineStr">
         <is>
           <t>Fare source (provenance)</t>
         </is>
       </c>
-      <c r="AY3" s="24" t="inlineStr">
+      <c r="AY3" s="25" t="inlineStr">
         <is>
           <t>Demand source (provenance)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="32" t="inlineStr">
         <is>
           <t>Jeddah Corniche → Jeddah Central (PIF waterfront)</t>
         </is>
       </c>
-      <c r="D4" s="31" t="n">
+      <c r="D4" s="33" t="n">
         <v>2.4</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="27" t="n">
         <v>60</v>
       </c>
-      <c r="F4" s="32" t="inlineStr">
+      <c r="F4" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G4" s="32" t="inlineStr">
+      <c r="G4" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="33">
+      <c r="I4" s="35">
         <f>60*D4/cruise_kt</f>
         <v/>
       </c>
-      <c r="J4" s="33">
+      <c r="J4" s="35">
         <f>I4+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K4" s="34">
+      <c r="K4" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J4,1))</f>
         <v/>
       </c>
-      <c r="L4" s="34">
-        <f>ROUND(365*mech_uptime*H4,0)</f>
-        <v/>
-      </c>
-      <c r="M4" s="35">
+      <c r="L4" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H4)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H4)/2,0),ROUND((365*mech_uptime*H4),0))</f>
+        <v/>
+      </c>
+      <c r="M4" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N4" s="35">
+      <c r="N4" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O4" s="34">
-        <f>ROUND(K4*L4*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P4" s="36">
+      <c r="O4" s="36">
+        <f>IF(ABS(MOD(ABS((K4*L4*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_sel)/2,0),ROUND((K4*L4*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P4" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q4" s="36">
+      <c r="Q4" s="38">
         <f>pax_cap*P4</f>
         <v/>
       </c>
-      <c r="R4" s="34">
+      <c r="R4" s="36">
         <f>Q4*O4</f>
         <v/>
       </c>
-      <c r="S4" s="37">
+      <c r="S4" s="39">
         <f>E4*discount</f>
         <v/>
       </c>
-      <c r="T4" s="38">
+      <c r="T4" s="40">
         <f>S4*R4</f>
         <v/>
       </c>
-      <c r="U4" s="38">
+      <c r="U4" s="40">
         <f>(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V4" s="38">
+      <c r="V4" s="40">
         <f>VLOOKUP(B4,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W4" s="38">
+      <c r="W4" s="40">
         <f>VLOOKUP(B4,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X4" s="38">
+      <c r="X4" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y4" s="38">
+      <c r="Y4" s="40">
         <f>VLOOKUP(B4,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z4" s="38">
+      <c r="Z4" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA4" s="38">
+      <c r="AA4" s="40">
         <f>U4+V4+W4+X4+Y4+Z4</f>
         <v/>
       </c>
-      <c r="AB4" s="38">
+      <c r="AB4" s="40">
         <f>VLOOKUP(B4,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC4" s="38">
+      <c r="AC4" s="40">
         <f>T4-AA4</f>
         <v/>
       </c>
-      <c r="AD4" s="35">
+      <c r="AD4" s="37">
         <f>IF(T4=0,"",AC4/T4)</f>
         <v/>
       </c>
-      <c r="AE4" s="36">
+      <c r="AE4" s="38">
         <f>IF(AC4&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/AC4)</f>
         <v/>
       </c>
-      <c r="AF4" s="33">
+      <c r="AF4" s="35">
         <f>((D4*O4/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG4" s="31" t="n"/>
-      <c r="AH4" s="32" t="inlineStr">
+      <c r="AG4" s="33" t="n"/>
+      <c r="AH4" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="AI4" s="32" t="inlineStr">
+      <c r="AI4" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="AJ4" s="39" t="n">
+      <c r="AJ4" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK4" s="34">
+      <c r="AK4" s="36">
         <f>IF(AG4="","",AG4*AJ4)</f>
         <v/>
       </c>
-      <c r="AL4" s="34">
+      <c r="AL4" s="36">
         <f>IF(OR(AG4="",R4=0),"",MIN(IF(AT4="",9.9E+99,AT4),FLOOR(AK4/R4,1)))</f>
         <v/>
       </c>
-      <c r="AM4" s="38">
-        <f>IF(AL4="","",AL4*T4)</f>
-        <v/>
-      </c>
-      <c r="AN4" s="36">
+      <c r="AM4" s="40">
+        <f>IF(AL4="","",AL4*IF(ABS(MOD(ABS((T4)),1)-0.5)&lt;1E-9,2*ROUND((T4)/2,0),ROUND((T4),0)))</f>
+        <v/>
+      </c>
+      <c r="AN4" s="38">
         <f>IF(OR(AG4="",R4=0),"",MIN(IF(AT4="",9.9E+99,AT4),AK4/R4))</f>
         <v/>
       </c>
-      <c r="AO4" s="38">
+      <c r="AO4" s="40">
         <f>IF(AN4="","",AN4*T4)</f>
         <v/>
       </c>
-      <c r="AP4" s="40" t="n"/>
-      <c r="AQ4" s="32" t="inlineStr">
+      <c r="AP4" s="42" t="n"/>
+      <c r="AQ4" s="34" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
-      <c r="AR4" s="41" t="n"/>
-      <c r="AS4" s="41" t="n"/>
-      <c r="AT4" s="42" t="n"/>
-      <c r="AU4" s="43">
-        <f>IF(((S4*pax_cap*load_thin*ROUND(K4*L4*revleg_thin,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_thin,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_thin*ROUND(K4*L4*revleg_thin,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_thin,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
-        <v/>
-      </c>
-      <c r="AV4" s="43">
-        <f>IF(((S4*pax_cap*load_mid*ROUND(K4*L4*revleg_mid,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_mid,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_mid*ROUND(K4*L4*revleg_mid,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_mid,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
-        <v/>
-      </c>
-      <c r="AW4" s="43">
-        <f>IF(((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
-        <v/>
-      </c>
-      <c r="AX4" s="44" t="inlineStr">
+      <c r="AR4" s="43" t="n"/>
+      <c r="AS4" s="43" t="n"/>
+      <c r="AT4" s="44" t="n"/>
+      <c r="AU4" s="45">
+        <f>IF(((S4*pax_cap*load_thin*IF(ABS(MOD(ABS((K4*L4*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_thin)/2,0),ROUND((K4*L4*revleg_thin),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_thin)/2,0),ROUND((K4*L4*revleg_thin),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_thin*IF(ABS(MOD(ABS((K4*L4*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_thin)/2,0),ROUND((K4*L4*revleg_thin),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_thin)/2,0),ROUND((K4*L4*revleg_thin),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
+        <v/>
+      </c>
+      <c r="AV4" s="45">
+        <f>IF(((S4*pax_cap*load_mid*IF(ABS(MOD(ABS((K4*L4*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_mid)/2,0),ROUND((K4*L4*revleg_mid),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_mid)/2,0),ROUND((K4*L4*revleg_mid),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_mid*IF(ABS(MOD(ABS((K4*L4*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_mid)/2,0),ROUND((K4*L4*revleg_mid),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_mid)/2,0),ROUND((K4*L4*revleg_mid),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
+        <v/>
+      </c>
+      <c r="AW4" s="45">
+        <f>IF(((S4*pax_cap*load_full*IF(ABS(MOD(ABS((K4*L4*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_full)/2,0),ROUND((K4*L4*revleg_full),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_full)/2,0),ROUND((K4*L4*revleg_full),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_full*IF(ABS(MOD(ABS((K4*L4*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_full)/2,0),ROUND((K4*L4*revleg_full),0)))-(((battery/range_nm)*D4*IF(ABS(MOD(ABS((K4*L4*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K4*L4*revleg_full)/2,0),ROUND((K4*L4*revleg_full),0))*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
+        <v/>
+      </c>
+      <c r="AX4" s="46" t="inlineStr">
         <is>
           <t>Premium urban/coastal water-transfer comparable (Dubai/Gulf premium water-taxi tier ~$40-80/pax). Jeddah Central is a $20B PIF waterfront (5.7km2, marina/oceanarium/beaches, opening ~2027). No incumbent water transit -&gt; modeled premium per-seat $60.</t>
         </is>
       </c>
-      <c r="AY4" s="44" t="inlineStr">
+      <c r="AY4" s="46" t="inlineStr">
         <is>
           <t>NULL (R2). No published Jeddah Central on-corridor / water-transit visitor target. Saudi national arrivals (100M 2024, target 150M 2030) and Jeddah city arrivals are AIR/ROAD-based (R3 strong mode mismatch) -&gt; not on-water crossing ridership. ALSO R6 FLAG: 45nm is geographically implausible for an intra-Jeddah Corniche&lt;-&gt;Jeddah Central waterfront hop (~few km apart) - likely a distance/routing artifact; report to parent.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Outer-island resort → Outer-island resort cluster (Nujuma / Jumeirah / St Regis)</t>
         </is>
       </c>
-      <c r="D5" s="31" t="n">
+      <c r="D5" s="33" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="27" t="n">
         <v>125</v>
       </c>
-      <c r="F5" s="32" t="inlineStr">
+      <c r="F5" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G5" s="32" t="inlineStr">
+      <c r="G5" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="33">
+      <c r="I5" s="35">
         <f>60*D5/cruise_kt</f>
         <v/>
       </c>
-      <c r="J5" s="33">
+      <c r="J5" s="35">
         <f>I5+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K5" s="34">
+      <c r="K5" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J5,1))</f>
         <v/>
       </c>
-      <c r="L5" s="34">
-        <f>ROUND(365*mech_uptime*H5,0)</f>
-        <v/>
-      </c>
-      <c r="M5" s="35">
+      <c r="L5" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H5)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H5)/2,0),ROUND((365*mech_uptime*H5),0))</f>
+        <v/>
+      </c>
+      <c r="M5" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N5" s="35">
+      <c r="N5" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O5" s="34">
-        <f>ROUND(K5*L5*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P5" s="36">
+      <c r="O5" s="36">
+        <f>IF(ABS(MOD(ABS((K5*L5*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_sel)/2,0),ROUND((K5*L5*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P5" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q5" s="36">
+      <c r="Q5" s="38">
         <f>pax_cap*P5</f>
         <v/>
       </c>
-      <c r="R5" s="34">
+      <c r="R5" s="36">
         <f>Q5*O5</f>
         <v/>
       </c>
-      <c r="S5" s="37">
+      <c r="S5" s="39">
         <f>E5*discount</f>
         <v/>
       </c>
-      <c r="T5" s="38">
+      <c r="T5" s="40">
         <f>S5*R5</f>
         <v/>
       </c>
-      <c r="U5" s="38">
+      <c r="U5" s="40">
         <f>(battery/range_nm)*D5*O5*VLOOKUP(B5,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V5" s="38">
+      <c r="V5" s="40">
         <f>VLOOKUP(B5,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W5" s="38">
+      <c r="W5" s="40">
         <f>VLOOKUP(B5,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X5" s="38">
+      <c r="X5" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y5" s="38">
+      <c r="Y5" s="40">
         <f>VLOOKUP(B5,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z5" s="38">
+      <c r="Z5" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA5" s="38">
+      <c r="AA5" s="40">
         <f>U5+V5+W5+X5+Y5+Z5</f>
         <v/>
       </c>
-      <c r="AB5" s="38">
+      <c r="AB5" s="40">
         <f>VLOOKUP(B5,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC5" s="38">
+      <c r="AC5" s="40">
         <f>T5-AA5</f>
         <v/>
       </c>
-      <c r="AD5" s="35">
+      <c r="AD5" s="37">
         <f>IF(T5=0,"",AC5/T5)</f>
         <v/>
       </c>
-      <c r="AE5" s="36">
+      <c r="AE5" s="38">
         <f>IF(AC5&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/AC5)</f>
         <v/>
       </c>
-      <c r="AF5" s="33">
+      <c r="AF5" s="35">
         <f>((D5*O5/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D5*O5*VLOOKUP(B5,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG5" s="31" t="n">
+      <c r="AG5" s="33" t="n">
         <v>150000</v>
       </c>
-      <c r="AH5" s="32" t="inlineStr">
+      <c r="AH5" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="AI5" s="32" t="inlineStr">
+      <c r="AI5" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="AJ5" s="39" t="n">
+      <c r="AJ5" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK5" s="34">
+      <c r="AK5" s="36">
         <f>IF(AG5="","",AG5*AJ5)</f>
         <v/>
       </c>
-      <c r="AL5" s="34">
+      <c r="AL5" s="36">
         <f>IF(OR(AG5="",R5=0),"",MIN(IF(AT5="",9.9E+99,AT5),FLOOR(AK5/R5,1)))</f>
         <v/>
       </c>
-      <c r="AM5" s="38">
-        <f>IF(AL5="","",AL5*T5)</f>
-        <v/>
-      </c>
-      <c r="AN5" s="36">
+      <c r="AM5" s="40">
+        <f>IF(AL5="","",AL5*IF(ABS(MOD(ABS((T5)),1)-0.5)&lt;1E-9,2*ROUND((T5)/2,0),ROUND((T5),0)))</f>
+        <v/>
+      </c>
+      <c r="AN5" s="38">
         <f>IF(OR(AG5="",R5=0),"",MIN(IF(AT5="",9.9E+99,AT5),AK5/R5))</f>
         <v/>
       </c>
-      <c r="AO5" s="38">
+      <c r="AO5" s="40">
         <f>IF(AN5="","",AN5*T5)</f>
         <v/>
       </c>
-      <c r="AP5" s="40" t="n"/>
-      <c r="AQ5" s="32" t="inlineStr">
+      <c r="AP5" s="42" t="n"/>
+      <c r="AQ5" s="34" t="inlineStr">
         <is>
           <t>Forward SAM</t>
         </is>
       </c>
-      <c r="AR5" s="41" t="inlineStr">
+      <c r="AR5" s="43" t="inlineStr">
         <is>
           <t>FWD-SAM (2030)</t>
         </is>
       </c>
-      <c r="AS5" s="41" t="n"/>
-      <c r="AT5" s="42" t="n"/>
-      <c r="AU5" s="43">
-        <f>IF(((S5*pax_cap*load_thin*ROUND(K5*L5*revleg_thin,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_thin,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_thin*ROUND(K5*L5*revleg_thin,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_thin,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
-        <v/>
-      </c>
-      <c r="AV5" s="43">
-        <f>IF(((S5*pax_cap*load_mid*ROUND(K5*L5*revleg_mid,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_mid,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_mid*ROUND(K5*L5*revleg_mid,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_mid,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
-        <v/>
-      </c>
-      <c r="AW5" s="43">
-        <f>IF(((S5*pax_cap*load_full*ROUND(K5*L5*revleg_full,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_full,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_full*ROUND(K5*L5*revleg_full,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_full,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
-        <v/>
-      </c>
-      <c r="AX5" s="44" t="inlineStr">
+      <c r="AS5" s="43" t="n"/>
+      <c r="AT5" s="44" t="n"/>
+      <c r="AU5" s="45">
+        <f>IF(((S5*pax_cap*load_thin*IF(ABS(MOD(ABS((K5*L5*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_thin)/2,0),ROUND((K5*L5*revleg_thin),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_thin)/2,0),ROUND((K5*L5*revleg_thin),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_thin*IF(ABS(MOD(ABS((K5*L5*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_thin)/2,0),ROUND((K5*L5*revleg_thin),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_thin)/2,0),ROUND((K5*L5*revleg_thin),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
+        <v/>
+      </c>
+      <c r="AV5" s="45">
+        <f>IF(((S5*pax_cap*load_mid*IF(ABS(MOD(ABS((K5*L5*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_mid)/2,0),ROUND((K5*L5*revleg_mid),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_mid)/2,0),ROUND((K5*L5*revleg_mid),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_mid*IF(ABS(MOD(ABS((K5*L5*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_mid)/2,0),ROUND((K5*L5*revleg_mid),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_mid)/2,0),ROUND((K5*L5*revleg_mid),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
+        <v/>
+      </c>
+      <c r="AW5" s="45">
+        <f>IF(((S5*pax_cap*load_full*IF(ABS(MOD(ABS((K5*L5*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_full)/2,0),ROUND((K5*L5*revleg_full),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_full)/2,0),ROUND((K5*L5*revleg_full),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_full*IF(ABS(MOD(ABS((K5*L5*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_full)/2,0),ROUND((K5*L5*revleg_full),0)))-(((battery/range_nm)*D5*IF(ABS(MOD(ABS((K5*L5*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K5*L5*revleg_full)/2,0),ROUND((K5*L5*revleg_full),0))*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
+        <v/>
+      </c>
+      <c r="AX5" s="46" t="inlineStr">
         <is>
           <t>Maldives resort speedboat transfer per-seat comparable (no incumbent on this greenfield Red Sea crossing, R5): MaldivesNomad resort transfers $65-350/pax 1-way; AtollTransfer $90-450/pax; premium private-resort $150-250 1-way; PointsGuy Marriott speedboat $142 RT. Premium per-seat point picked. 12nm short intra-resort island hop -&gt; premium per-seat $125.</t>
         </is>
       </c>
-      <c r="AY5" s="44" t="inlineStr">
+      <c r="AY5" s="46" t="inlineStr">
         <is>
           <t>Subset of RSG 1M/yr visitor cap doing outer-island-to-outer-island hops (not the main arrival leg). Modeled ~15% of the 1M pool ~150k. Speculative which guests hop islands; R2 borderline.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>Shura Island Marina → Outer-island resorts (St Regis / Nujuma / Shebara)</t>
         </is>
       </c>
-      <c r="D6" s="31" t="n">
+      <c r="D6" s="33" t="n">
         <v>11.5</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="27" t="n">
         <v>175</v>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="G6" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="33">
+      <c r="I6" s="35">
         <f>60*D6/cruise_kt</f>
         <v/>
       </c>
-      <c r="J6" s="33">
+      <c r="J6" s="35">
         <f>I6+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J6,1))</f>
         <v/>
       </c>
-      <c r="L6" s="34">
-        <f>ROUND(365*mech_uptime*H6,0)</f>
-        <v/>
-      </c>
-      <c r="M6" s="35">
+      <c r="L6" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H6)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H6)/2,0),ROUND((365*mech_uptime*H6),0))</f>
+        <v/>
+      </c>
+      <c r="M6" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N6" s="35">
+      <c r="N6" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O6" s="34">
-        <f>ROUND(K6*L6*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P6" s="36">
+      <c r="O6" s="36">
+        <f>IF(ABS(MOD(ABS((K6*L6*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_sel)/2,0),ROUND((K6*L6*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P6" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q6" s="36">
+      <c r="Q6" s="38">
         <f>pax_cap*P6</f>
         <v/>
       </c>
-      <c r="R6" s="34">
+      <c r="R6" s="36">
         <f>Q6*O6</f>
         <v/>
       </c>
-      <c r="S6" s="37">
+      <c r="S6" s="39">
         <f>E6*discount</f>
         <v/>
       </c>
-      <c r="T6" s="38">
+      <c r="T6" s="40">
         <f>S6*R6</f>
         <v/>
       </c>
-      <c r="U6" s="38">
+      <c r="U6" s="40">
         <f>(battery/range_nm)*D6*O6*VLOOKUP(B6,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V6" s="38">
+      <c r="V6" s="40">
         <f>VLOOKUP(B6,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W6" s="38">
+      <c r="W6" s="40">
         <f>VLOOKUP(B6,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X6" s="38">
+      <c r="X6" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y6" s="38">
+      <c r="Y6" s="40">
         <f>VLOOKUP(B6,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z6" s="38">
+      <c r="Z6" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA6" s="38">
+      <c r="AA6" s="40">
         <f>U6+V6+W6+X6+Y6+Z6</f>
         <v/>
       </c>
-      <c r="AB6" s="38">
+      <c r="AB6" s="40">
         <f>VLOOKUP(B6,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC6" s="38">
+      <c r="AC6" s="40">
         <f>T6-AA6</f>
         <v/>
       </c>
-      <c r="AD6" s="35">
+      <c r="AD6" s="37">
         <f>IF(T6=0,"",AC6/T6)</f>
         <v/>
       </c>
-      <c r="AE6" s="36">
+      <c r="AE6" s="38">
         <f>IF(AC6&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/AC6)</f>
         <v/>
       </c>
-      <c r="AF6" s="33">
+      <c r="AF6" s="35">
         <f>((D6*O6/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D6*O6*VLOOKUP(B6,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG6" s="31" t="n">
+      <c r="AG6" s="33" t="n">
         <v>500000</v>
       </c>
-      <c r="AH6" s="32" t="inlineStr">
+      <c r="AH6" s="34" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="AI6" s="32" t="inlineStr">
+      <c r="AI6" s="34" t="inlineStr">
         <is>
           <t>low-med</t>
         </is>
       </c>
-      <c r="AJ6" s="39" t="n">
+      <c r="AJ6" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK6" s="34">
+      <c r="AK6" s="36">
         <f>IF(AG6="","",AG6*AJ6)</f>
         <v/>
       </c>
-      <c r="AL6" s="34">
+      <c r="AL6" s="36">
         <f>IF(OR(AG6="",R6=0),"",MIN(IF(AT6="",9.9E+99,AT6),FLOOR(AK6/R6,1)))</f>
         <v/>
       </c>
-      <c r="AM6" s="38">
-        <f>IF(AL6="","",AL6*T6)</f>
-        <v/>
-      </c>
-      <c r="AN6" s="36">
+      <c r="AM6" s="40">
+        <f>IF(AL6="","",AL6*IF(ABS(MOD(ABS((T6)),1)-0.5)&lt;1E-9,2*ROUND((T6)/2,0),ROUND((T6),0)))</f>
+        <v/>
+      </c>
+      <c r="AN6" s="38">
         <f>IF(OR(AG6="",R6=0),"",MIN(IF(AT6="",9.9E+99,AT6),AK6/R6))</f>
         <v/>
       </c>
-      <c r="AO6" s="38">
+      <c r="AO6" s="40">
         <f>IF(AN6="","",AN6*T6)</f>
         <v/>
       </c>
-      <c r="AP6" s="40" t="n"/>
-      <c r="AQ6" s="32" t="inlineStr">
+      <c r="AP6" s="42" t="n"/>
+      <c r="AQ6" s="34" t="inlineStr">
         <is>
           <t>Forward SAM</t>
         </is>
       </c>
-      <c r="AR6" s="41" t="inlineStr">
+      <c r="AR6" s="43" t="inlineStr">
         <is>
           <t>FWD-SAM (2030)</t>
         </is>
       </c>
-      <c r="AS6" s="41" t="n"/>
-      <c r="AT6" s="42" t="n"/>
-      <c r="AU6" s="43">
-        <f>IF(((S6*pax_cap*load_thin*ROUND(K6*L6*revleg_thin,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_thin,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_thin*ROUND(K6*L6*revleg_thin,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_thin,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
-        <v/>
-      </c>
-      <c r="AV6" s="43">
-        <f>IF(((S6*pax_cap*load_mid*ROUND(K6*L6*revleg_mid,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_mid,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_mid*ROUND(K6*L6*revleg_mid,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_mid,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
-        <v/>
-      </c>
-      <c r="AW6" s="43">
-        <f>IF(((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
-        <v/>
-      </c>
-      <c r="AX6" s="44" t="inlineStr">
+      <c r="AS6" s="43" t="n"/>
+      <c r="AT6" s="44" t="n"/>
+      <c r="AU6" s="45">
+        <f>IF(((S6*pax_cap*load_thin*IF(ABS(MOD(ABS((K6*L6*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_thin)/2,0),ROUND((K6*L6*revleg_thin),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_thin)/2,0),ROUND((K6*L6*revleg_thin),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_thin*IF(ABS(MOD(ABS((K6*L6*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_thin)/2,0),ROUND((K6*L6*revleg_thin),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_thin)/2,0),ROUND((K6*L6*revleg_thin),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
+        <v/>
+      </c>
+      <c r="AV6" s="45">
+        <f>IF(((S6*pax_cap*load_mid*IF(ABS(MOD(ABS((K6*L6*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_mid)/2,0),ROUND((K6*L6*revleg_mid),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_mid)/2,0),ROUND((K6*L6*revleg_mid),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_mid*IF(ABS(MOD(ABS((K6*L6*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_mid)/2,0),ROUND((K6*L6*revleg_mid),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_mid)/2,0),ROUND((K6*L6*revleg_mid),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
+        <v/>
+      </c>
+      <c r="AW6" s="45">
+        <f>IF(((S6*pax_cap*load_full*IF(ABS(MOD(ABS((K6*L6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_full)/2,0),ROUND((K6*L6*revleg_full),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_full)/2,0),ROUND((K6*L6*revleg_full),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_full*IF(ABS(MOD(ABS((K6*L6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_full)/2,0),ROUND((K6*L6*revleg_full),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((K6*L6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K6*L6*revleg_full)/2,0),ROUND((K6*L6*revleg_full),0))*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
+        <v/>
+      </c>
+      <c r="AX6" s="46" t="inlineStr">
         <is>
           <t>Maldives resort speedboat transfer per-seat comparable (no incumbent on this greenfield Red Sea crossing, R5): MaldivesNomad resort transfers $65-350/pax 1-way; AtollTransfer $90-450/pax; premium private-resort $150-250 1-way; PointsGuy Marriott speedboat $142 RT. Premium per-seat point picked. 25nm outer-island luxury resort transfer -&gt; premium per-seat $175.</t>
         </is>
       </c>
-      <c r="AY6" s="44" t="inlineStr">
+      <c r="AY6" s="46" t="inlineStr">
         <is>
           <t>Red Sea Global / The Red Sea destination capped at 1,000,000 visitors/yr at full completion 2030 across 50 resorts/8,000+ keys (RSG official; Monaco Yacht Show factsheet 2025; blooloop; ICWA). Shura Island hub-&gt;outer-island resorts is THE primary internal transfer leg; R3 discount ~50% (not all resorts outer-island; some mainland/nearshore) -&gt; ~500k 1-way.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>Jeddah Corniche → Jeddah Yacht Club &amp; Marina</t>
         </is>
       </c>
-      <c r="D7" s="31" t="n">
+      <c r="D7" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="E7" s="26" t="n"/>
-      <c r="F7" s="32" t="n"/>
-      <c r="G7" s="32" t="n"/>
-      <c r="H7" s="19" t="n">
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="34" t="n"/>
+      <c r="G7" s="34" t="n"/>
+      <c r="H7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="33">
+      <c r="I7" s="35">
         <f>60*D7/cruise_kt</f>
         <v/>
       </c>
-      <c r="J7" s="33">
+      <c r="J7" s="35">
         <f>I7+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K7" s="34">
+      <c r="K7" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J7,1))</f>
         <v/>
       </c>
-      <c r="L7" s="34">
-        <f>ROUND(365*mech_uptime*H7,0)</f>
-        <v/>
-      </c>
-      <c r="M7" s="35">
+      <c r="L7" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H7)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H7)/2,0),ROUND((365*mech_uptime*H7),0))</f>
+        <v/>
+      </c>
+      <c r="M7" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N7" s="35">
+      <c r="N7" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O7" s="34">
-        <f>ROUND(K7*L7*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P7" s="36">
+      <c r="O7" s="36">
+        <f>IF(ABS(MOD(ABS((K7*L7*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_sel)/2,0),ROUND((K7*L7*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P7" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q7" s="36">
+      <c r="Q7" s="38">
         <f>pax_cap*P7</f>
         <v/>
       </c>
-      <c r="R7" s="34">
+      <c r="R7" s="36">
         <f>Q7*O7</f>
         <v/>
       </c>
-      <c r="S7" s="37">
+      <c r="S7" s="39">
         <f>E7*discount</f>
         <v/>
       </c>
-      <c r="T7" s="38">
+      <c r="T7" s="40">
         <f>S7*R7</f>
         <v/>
       </c>
-      <c r="U7" s="38">
+      <c r="U7" s="40">
         <f>(battery/range_nm)*D7*O7*VLOOKUP(B7,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V7" s="38">
+      <c r="V7" s="40">
         <f>VLOOKUP(B7,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W7" s="38">
+      <c r="W7" s="40">
         <f>VLOOKUP(B7,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X7" s="38">
+      <c r="X7" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y7" s="38">
+      <c r="Y7" s="40">
         <f>VLOOKUP(B7,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z7" s="38">
+      <c r="Z7" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA7" s="38">
+      <c r="AA7" s="40">
         <f>U7+V7+W7+X7+Y7+Z7</f>
         <v/>
       </c>
-      <c r="AB7" s="38">
+      <c r="AB7" s="40">
         <f>VLOOKUP(B7,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC7" s="38">
+      <c r="AC7" s="40">
         <f>T7-AA7</f>
         <v/>
       </c>
-      <c r="AD7" s="35">
+      <c r="AD7" s="37">
         <f>IF(T7=0,"",AC7/T7)</f>
         <v/>
       </c>
-      <c r="AE7" s="36">
+      <c r="AE7" s="38">
         <f>IF(AC7&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/AC7)</f>
         <v/>
       </c>
-      <c r="AF7" s="33">
+      <c r="AF7" s="35">
         <f>((D7*O7/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D7*O7*VLOOKUP(B7,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG7" s="31" t="n"/>
-      <c r="AH7" s="32" t="n"/>
-      <c r="AI7" s="32" t="n"/>
-      <c r="AJ7" s="39" t="n">
+      <c r="AG7" s="33" t="n"/>
+      <c r="AH7" s="34" t="n"/>
+      <c r="AI7" s="34" t="n"/>
+      <c r="AJ7" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK7" s="34">
+      <c r="AK7" s="36">
         <f>IF(AG7="","",AG7*AJ7)</f>
         <v/>
       </c>
-      <c r="AL7" s="34">
+      <c r="AL7" s="36">
         <f>IF(OR(AG7="",R7=0),"",MIN(IF(AT7="",9.9E+99,AT7),FLOOR(AK7/R7,1)))</f>
         <v/>
       </c>
-      <c r="AM7" s="38">
-        <f>IF(AL7="","",AL7*T7)</f>
-        <v/>
-      </c>
-      <c r="AN7" s="36">
+      <c r="AM7" s="40">
+        <f>IF(AL7="","",AL7*IF(ABS(MOD(ABS((T7)),1)-0.5)&lt;1E-9,2*ROUND((T7)/2,0),ROUND((T7),0)))</f>
+        <v/>
+      </c>
+      <c r="AN7" s="38">
         <f>IF(OR(AG7="",R7=0),"",MIN(IF(AT7="",9.9E+99,AT7),AK7/R7))</f>
         <v/>
       </c>
-      <c r="AO7" s="38">
+      <c r="AO7" s="40">
         <f>IF(AN7="","",AN7*T7)</f>
         <v/>
       </c>
-      <c r="AP7" s="40" t="n"/>
-      <c r="AQ7" s="32" t="inlineStr">
+      <c r="AP7" s="42" t="n"/>
+      <c r="AQ7" s="34" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
-      <c r="AR7" s="41" t="n"/>
-      <c r="AS7" s="41" t="n"/>
-      <c r="AT7" s="42" t="n"/>
-      <c r="AU7" s="43">
-        <f>IF(((S7*pax_cap*load_thin*ROUND(K7*L7*revleg_thin,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_thin,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_thin*ROUND(K7*L7*revleg_thin,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_thin,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
-        <v/>
-      </c>
-      <c r="AV7" s="43">
-        <f>IF(((S7*pax_cap*load_mid*ROUND(K7*L7*revleg_mid,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_mid,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_mid*ROUND(K7*L7*revleg_mid,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_mid,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
-        <v/>
-      </c>
-      <c r="AW7" s="43">
-        <f>IF(((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
-        <v/>
-      </c>
-      <c r="AX7" s="44" t="n"/>
-      <c r="AY7" s="44" t="n"/>
+      <c r="AR7" s="43" t="n"/>
+      <c r="AS7" s="43" t="n"/>
+      <c r="AT7" s="44" t="n"/>
+      <c r="AU7" s="45">
+        <f>IF(((S7*pax_cap*load_thin*IF(ABS(MOD(ABS((K7*L7*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_thin)/2,0),ROUND((K7*L7*revleg_thin),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_thin)/2,0),ROUND((K7*L7*revleg_thin),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_thin*IF(ABS(MOD(ABS((K7*L7*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_thin)/2,0),ROUND((K7*L7*revleg_thin),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_thin)/2,0),ROUND((K7*L7*revleg_thin),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
+        <v/>
+      </c>
+      <c r="AV7" s="45">
+        <f>IF(((S7*pax_cap*load_mid*IF(ABS(MOD(ABS((K7*L7*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_mid)/2,0),ROUND((K7*L7*revleg_mid),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_mid)/2,0),ROUND((K7*L7*revleg_mid),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_mid*IF(ABS(MOD(ABS((K7*L7*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_mid)/2,0),ROUND((K7*L7*revleg_mid),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_mid)/2,0),ROUND((K7*L7*revleg_mid),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
+        <v/>
+      </c>
+      <c r="AW7" s="45">
+        <f>IF(((S7*pax_cap*load_full*IF(ABS(MOD(ABS((K7*L7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_full)/2,0),ROUND((K7*L7*revleg_full),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_full)/2,0),ROUND((K7*L7*revleg_full),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_full*IF(ABS(MOD(ABS((K7*L7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_full)/2,0),ROUND((K7*L7*revleg_full),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((K7*L7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K7*L7*revleg_full)/2,0),ROUND((K7*L7*revleg_full),0))*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
+        <v/>
+      </c>
+      <c r="AX7" s="46" t="n"/>
+      <c r="AY7" s="46" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>Khobar / Dammam (Eastern Province) → Manama, Bahrain</t>
         </is>
       </c>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="33" t="n">
         <v>18.6</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="27" t="n">
         <v>80</v>
       </c>
-      <c r="F8" s="32" t="inlineStr">
+      <c r="F8" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G8" s="32" t="inlineStr">
+      <c r="G8" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="33">
+      <c r="I8" s="35">
         <f>60*D8/cruise_kt</f>
         <v/>
       </c>
-      <c r="J8" s="33">
+      <c r="J8" s="35">
         <f>I8+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J8,1))</f>
         <v/>
       </c>
-      <c r="L8" s="34">
-        <f>ROUND(365*mech_uptime*H8,0)</f>
-        <v/>
-      </c>
-      <c r="M8" s="35">
+      <c r="L8" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H8)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H8)/2,0),ROUND((365*mech_uptime*H8),0))</f>
+        <v/>
+      </c>
+      <c r="M8" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N8" s="35">
+      <c r="N8" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O8" s="34">
-        <f>ROUND(K8*L8*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P8" s="36">
+      <c r="O8" s="36">
+        <f>IF(ABS(MOD(ABS((K8*L8*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_sel)/2,0),ROUND((K8*L8*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P8" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q8" s="36">
+      <c r="Q8" s="38">
         <f>pax_cap*P8</f>
         <v/>
       </c>
-      <c r="R8" s="34">
+      <c r="R8" s="36">
         <f>Q8*O8</f>
         <v/>
       </c>
-      <c r="S8" s="37">
+      <c r="S8" s="39">
         <f>E8*discount</f>
         <v/>
       </c>
-      <c r="T8" s="38">
+      <c r="T8" s="40">
         <f>S8*R8</f>
         <v/>
       </c>
-      <c r="U8" s="38">
+      <c r="U8" s="40">
         <f>(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V8" s="38">
+      <c r="V8" s="40">
         <f>VLOOKUP(B8,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W8" s="38">
+      <c r="W8" s="40">
         <f>VLOOKUP(B8,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X8" s="38">
+      <c r="X8" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y8" s="38">
+      <c r="Y8" s="40">
         <f>VLOOKUP(B8,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z8" s="38">
+      <c r="Z8" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA8" s="38">
+      <c r="AA8" s="40">
         <f>U8+V8+W8+X8+Y8+Z8</f>
         <v/>
       </c>
-      <c r="AB8" s="38">
+      <c r="AB8" s="40">
         <f>VLOOKUP(B8,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC8" s="38">
+      <c r="AC8" s="40">
         <f>T8-AA8</f>
         <v/>
       </c>
-      <c r="AD8" s="35">
+      <c r="AD8" s="37">
         <f>IF(T8=0,"",AC8/T8)</f>
         <v/>
       </c>
-      <c r="AE8" s="36">
+      <c r="AE8" s="38">
         <f>IF(AC8&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/AC8)</f>
         <v/>
       </c>
-      <c r="AF8" s="33">
+      <c r="AF8" s="35">
         <f>((D8*O8/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG8" s="31" t="n">
+      <c r="AG8" s="33" t="n">
         <v>330000</v>
       </c>
-      <c r="AH8" s="32" t="inlineStr">
+      <c r="AH8" s="34" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="AI8" s="32" t="inlineStr">
+      <c r="AI8" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="AJ8" s="39" t="n">
+      <c r="AJ8" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK8" s="34">
+      <c r="AK8" s="36">
         <f>IF(AG8="","",AG8*AJ8)</f>
         <v/>
       </c>
-      <c r="AL8" s="34">
+      <c r="AL8" s="36">
         <f>IF(OR(AG8="",R8=0),"",MIN(IF(AT8="",9.9E+99,AT8),FLOOR(AK8/R8,1)))</f>
         <v/>
       </c>
-      <c r="AM8" s="38">
-        <f>IF(AL8="","",AL8*T8)</f>
-        <v/>
-      </c>
-      <c r="AN8" s="36">
+      <c r="AM8" s="40">
+        <f>IF(AL8="","",AL8*IF(ABS(MOD(ABS((T8)),1)-0.5)&lt;1E-9,2*ROUND((T8)/2,0),ROUND((T8),0)))</f>
+        <v/>
+      </c>
+      <c r="AN8" s="38">
         <f>IF(OR(AG8="",R8=0),"",MIN(IF(AT8="",9.9E+99,AT8),AK8/R8))</f>
         <v/>
       </c>
-      <c r="AO8" s="38">
+      <c r="AO8" s="40">
         <f>IF(AN8="","",AN8*T8)</f>
         <v/>
       </c>
-      <c r="AP8" s="40" t="n"/>
-      <c r="AQ8" s="32" t="inlineStr">
+      <c r="AP8" s="42" t="n"/>
+      <c r="AQ8" s="34" t="inlineStr">
         <is>
           <t>Grounded</t>
         </is>
       </c>
-      <c r="AR8" s="41" t="n"/>
-      <c r="AS8" s="41" t="n"/>
-      <c r="AT8" s="42" t="n"/>
-      <c r="AU8" s="43">
-        <f>IF(((S8*pax_cap*load_thin*ROUND(K8*L8*revleg_thin,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_thin,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_thin*ROUND(K8*L8*revleg_thin,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_thin,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
-        <v/>
-      </c>
-      <c r="AV8" s="43">
-        <f>IF(((S8*pax_cap*load_mid*ROUND(K8*L8*revleg_mid,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_mid,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_mid*ROUND(K8*L8*revleg_mid,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_mid,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
-        <v/>
-      </c>
-      <c r="AW8" s="43">
-        <f>IF(((S8*pax_cap*load_full*ROUND(K8*L8*revleg_full,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_full,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_full*ROUND(K8*L8*revleg_full,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_full,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
-        <v/>
-      </c>
-      <c r="AX8" s="44" t="inlineStr">
+      <c r="AR8" s="43" t="n"/>
+      <c r="AS8" s="43" t="n"/>
+      <c r="AT8" s="44" t="n"/>
+      <c r="AU8" s="45">
+        <f>IF(((S8*pax_cap*load_thin*IF(ABS(MOD(ABS((K8*L8*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_thin)/2,0),ROUND((K8*L8*revleg_thin),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_thin)/2,0),ROUND((K8*L8*revleg_thin),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_thin*IF(ABS(MOD(ABS((K8*L8*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_thin)/2,0),ROUND((K8*L8*revleg_thin),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_thin)/2,0),ROUND((K8*L8*revleg_thin),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
+        <v/>
+      </c>
+      <c r="AV8" s="45">
+        <f>IF(((S8*pax_cap*load_mid*IF(ABS(MOD(ABS((K8*L8*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_mid)/2,0),ROUND((K8*L8*revleg_mid),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_mid)/2,0),ROUND((K8*L8*revleg_mid),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_mid*IF(ABS(MOD(ABS((K8*L8*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_mid)/2,0),ROUND((K8*L8*revleg_mid),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_mid)/2,0),ROUND((K8*L8*revleg_mid),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
+        <v/>
+      </c>
+      <c r="AW8" s="45">
+        <f>IF(((S8*pax_cap*load_full*IF(ABS(MOD(ABS((K8*L8*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_full)/2,0),ROUND((K8*L8*revleg_full),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_full)/2,0),ROUND((K8*L8*revleg_full),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_full*IF(ABS(MOD(ABS((K8*L8*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_full)/2,0),ROUND((K8*L8*revleg_full),0)))-(((battery/range_nm)*D8*IF(ABS(MOD(ABS((K8*L8*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K8*L8*revleg_full)/2,0),ROUND((K8*L8*revleg_full),0))*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
+        <v/>
+      </c>
+      <c r="AX8" s="46" t="inlineStr">
         <is>
           <t>No passenger ferry on this 25nm cross-Gulf crossing today (everyone DRIVES the King Fahd Causeway). Premium per-seat cross-Gulf fast transfer modeled on Gulf premium intercity/business transfer tier -&gt; $80. R16 home-port opex = Saudi Arabia.</t>
         </is>
       </c>
-      <c r="AY8" s="44" t="inlineStr">
+      <c r="AY8" s="46" t="inlineStr">
         <is>
           <t>King Fahd Causeway carried a RECORD 33,000,000 passengers in 2024 (Gulf News; ~52,450/day, +7%/yr) - but that is ROAD traffic (R3 strong mode mismatch). Do NOT claim full causeway volume. Addressable premium MARINE subset only: modeled ~1% of 33M = ~330k/yr 1-way (time-sensitive premium travelers who'd pay for a fast boat vs causeway congestion).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>The Red Sea → AMAALA (Triple Bay)</t>
         </is>
       </c>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="33" t="n">
         <v>29.4</v>
       </c>
-      <c r="E9" s="26" t="n">
+      <c r="E9" s="27" t="n">
         <v>250</v>
       </c>
-      <c r="F9" s="32" t="inlineStr">
+      <c r="F9" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G9" s="32" t="inlineStr">
+      <c r="G9" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="33">
+      <c r="I9" s="35">
         <f>60*D9/cruise_kt</f>
         <v/>
       </c>
-      <c r="J9" s="33">
+      <c r="J9" s="35">
         <f>I9+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K9" s="34">
+      <c r="K9" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J9,1))</f>
         <v/>
       </c>
-      <c r="L9" s="34">
-        <f>ROUND(365*mech_uptime*H9,0)</f>
-        <v/>
-      </c>
-      <c r="M9" s="35">
+      <c r="L9" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H9)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H9)/2,0),ROUND((365*mech_uptime*H9),0))</f>
+        <v/>
+      </c>
+      <c r="M9" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N9" s="35">
+      <c r="N9" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O9" s="34">
-        <f>ROUND(K9*L9*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P9" s="36">
+      <c r="O9" s="36">
+        <f>IF(ABS(MOD(ABS((K9*L9*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_sel)/2,0),ROUND((K9*L9*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P9" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q9" s="36">
+      <c r="Q9" s="38">
         <f>pax_cap*P9</f>
         <v/>
       </c>
-      <c r="R9" s="34">
+      <c r="R9" s="36">
         <f>Q9*O9</f>
         <v/>
       </c>
-      <c r="S9" s="37">
+      <c r="S9" s="39">
         <f>E9*discount</f>
         <v/>
       </c>
-      <c r="T9" s="38">
+      <c r="T9" s="40">
         <f>S9*R9</f>
         <v/>
       </c>
-      <c r="U9" s="38">
+      <c r="U9" s="40">
         <f>(battery/range_nm)*D9*O9*VLOOKUP(B9,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V9" s="38">
+      <c r="V9" s="40">
         <f>VLOOKUP(B9,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W9" s="38">
+      <c r="W9" s="40">
         <f>VLOOKUP(B9,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X9" s="38">
+      <c r="X9" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y9" s="38">
+      <c r="Y9" s="40">
         <f>VLOOKUP(B9,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z9" s="38">
+      <c r="Z9" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA9" s="38">
+      <c r="AA9" s="40">
         <f>U9+V9+W9+X9+Y9+Z9</f>
         <v/>
       </c>
-      <c r="AB9" s="38">
+      <c r="AB9" s="40">
         <f>VLOOKUP(B9,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC9" s="38">
+      <c r="AC9" s="40">
         <f>T9-AA9</f>
         <v/>
       </c>
-      <c r="AD9" s="35">
+      <c r="AD9" s="37">
         <f>IF(T9=0,"",AC9/T9)</f>
         <v/>
       </c>
-      <c r="AE9" s="36">
+      <c r="AE9" s="38">
         <f>IF(AC9&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/AC9)</f>
         <v/>
       </c>
-      <c r="AF9" s="33">
+      <c r="AF9" s="35">
         <f>((D9*O9/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D9*O9*VLOOKUP(B9,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG9" s="31" t="n">
+      <c r="AG9" s="33" t="n">
         <v>500000</v>
       </c>
-      <c r="AH9" s="32" t="inlineStr">
+      <c r="AH9" s="34" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="AI9" s="32" t="inlineStr">
+      <c r="AI9" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="AJ9" s="39" t="n">
+      <c r="AJ9" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK9" s="34">
+      <c r="AK9" s="36">
         <f>IF(AG9="","",AG9*AJ9)</f>
         <v/>
       </c>
-      <c r="AL9" s="34">
+      <c r="AL9" s="36">
         <f>IF(OR(AG9="",R9=0),"",MIN(IF(AT9="",9.9E+99,AT9),FLOOR(AK9/R9,1)))</f>
         <v/>
       </c>
-      <c r="AM9" s="38">
-        <f>IF(AL9="","",AL9*T9)</f>
-        <v/>
-      </c>
-      <c r="AN9" s="36">
+      <c r="AM9" s="40">
+        <f>IF(AL9="","",AL9*IF(ABS(MOD(ABS((T9)),1)-0.5)&lt;1E-9,2*ROUND((T9)/2,0),ROUND((T9),0)))</f>
+        <v/>
+      </c>
+      <c r="AN9" s="38">
         <f>IF(OR(AG9="",R9=0),"",MIN(IF(AT9="",9.9E+99,AT9),AK9/R9))</f>
         <v/>
       </c>
-      <c r="AO9" s="38">
+      <c r="AO9" s="40">
         <f>IF(AN9="","",AN9*T9)</f>
         <v/>
       </c>
-      <c r="AP9" s="40" t="n"/>
-      <c r="AQ9" s="32" t="inlineStr">
+      <c r="AP9" s="42" t="n"/>
+      <c r="AQ9" s="34" t="inlineStr">
         <is>
           <t>Grounded</t>
         </is>
       </c>
-      <c r="AR9" s="41" t="n"/>
-      <c r="AS9" s="41" t="n"/>
-      <c r="AT9" s="42" t="n"/>
-      <c r="AU9" s="43">
-        <f>IF(((S9*pax_cap*load_thin*ROUND(K9*L9*revleg_thin,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_thin,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_thin*ROUND(K9*L9*revleg_thin,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_thin,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
-        <v/>
-      </c>
-      <c r="AV9" s="43">
-        <f>IF(((S9*pax_cap*load_mid*ROUND(K9*L9*revleg_mid,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_mid,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_mid*ROUND(K9*L9*revleg_mid,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_mid,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
-        <v/>
-      </c>
-      <c r="AW9" s="43">
-        <f>IF(((S9*pax_cap*load_full*ROUND(K9*L9*revleg_full,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_full,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_full*ROUND(K9*L9*revleg_full,0))-(((battery/range_nm)*D9*ROUND(K9*L9*revleg_full,0)*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
-        <v/>
-      </c>
-      <c r="AX9" s="44" t="inlineStr">
+      <c r="AR9" s="43" t="n"/>
+      <c r="AS9" s="43" t="n"/>
+      <c r="AT9" s="44" t="n"/>
+      <c r="AU9" s="45">
+        <f>IF(((S9*pax_cap*load_thin*IF(ABS(MOD(ABS((K9*L9*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_thin)/2,0),ROUND((K9*L9*revleg_thin),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_thin)/2,0),ROUND((K9*L9*revleg_thin),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_thin*IF(ABS(MOD(ABS((K9*L9*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_thin)/2,0),ROUND((K9*L9*revleg_thin),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_thin)/2,0),ROUND((K9*L9*revleg_thin),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
+        <v/>
+      </c>
+      <c r="AV9" s="45">
+        <f>IF(((S9*pax_cap*load_mid*IF(ABS(MOD(ABS((K9*L9*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_mid)/2,0),ROUND((K9*L9*revleg_mid),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_mid)/2,0),ROUND((K9*L9*revleg_mid),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_mid*IF(ABS(MOD(ABS((K9*L9*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_mid)/2,0),ROUND((K9*L9*revleg_mid),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_mid)/2,0),ROUND((K9*L9*revleg_mid),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
+        <v/>
+      </c>
+      <c r="AW9" s="45">
+        <f>IF(((S9*pax_cap*load_full*IF(ABS(MOD(ABS((K9*L9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_full)/2,0),ROUND((K9*L9*revleg_full),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_full)/2,0),ROUND((K9*L9*revleg_full),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((S9*pax_cap*load_full*IF(ABS(MOD(ABS((K9*L9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_full)/2,0),ROUND((K9*L9*revleg_full),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((K9*L9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K9*L9*revleg_full)/2,0),ROUND((K9*L9*revleg_full),0))*VLOOKUP(B9,country_opex,3,FALSE))+V9+W9+X9+Y9+Z9)))</f>
+        <v/>
+      </c>
+      <c r="AX9" s="46" t="inlineStr">
         <is>
           <t>80nm luxury inter-destination leg - flight/seaplane-substituted (R12). Anchored on Maldives seaplane tier ($300-600 RT ~ $200-300 1-way) -&gt; premium per-seat ~$250. Held-out Quanta-LR roadmap leg.</t>
         </is>
       </c>
-      <c r="AY9" s="44" t="inlineStr">
+      <c r="AY9" s="46" t="inlineStr">
         <is>
           <t>AMAALA target ~500k/yr (The Red Sea + AMAALA combined aim ~1.5M visitors/yr; The Red Sea =1M -&gt; AMAALA ~0.5M). AMAALA full completion ~3,900 keys / up to 29-30 resorts (Four Seasons/RSG). Inter-destination transfer is a small subset; recorded AMAALA pool proxy low conf. Held-out leg.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>NEOM — Sindalah → Magna / Oxagon coast</t>
         </is>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="33" t="n">
         <v>30.8</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="F10" s="32" t="inlineStr">
+      <c r="F10" s="34" t="inlineStr">
         <is>
           <t>T5</t>
         </is>
       </c>
-      <c r="G10" s="32" t="inlineStr">
+      <c r="G10" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="35">
         <f>60*D10/cruise_kt</f>
         <v/>
       </c>
-      <c r="J10" s="33">
+      <c r="J10" s="35">
         <f>I10+turn_min+dwell_min</f>
         <v/>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="36">
         <f>MIN(15,FLOOR(60*service_hr/J10,1))</f>
         <v/>
       </c>
-      <c r="L10" s="34">
-        <f>ROUND(365*mech_uptime*H10,0)</f>
-        <v/>
-      </c>
-      <c r="M10" s="35">
+      <c r="L10" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H10)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H10)/2,0),ROUND((365*mech_uptime*H10),0))</f>
+        <v/>
+      </c>
+      <c r="M10" s="37">
         <f>mech_uptime</f>
         <v/>
       </c>
-      <c r="N10" s="35">
+      <c r="N10" s="37">
         <f>revleg_sel</f>
         <v/>
       </c>
-      <c r="O10" s="34">
-        <f>ROUND(K10*L10*revleg_sel,0)</f>
-        <v/>
-      </c>
-      <c r="P10" s="36">
+      <c r="O10" s="36">
+        <f>IF(ABS(MOD(ABS((K10*L10*revleg_sel)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_sel)/2,0),ROUND((K10*L10*revleg_sel),0))</f>
+        <v/>
+      </c>
+      <c r="P10" s="38">
         <f>load_sel</f>
         <v/>
       </c>
-      <c r="Q10" s="36">
+      <c r="Q10" s="38">
         <f>pax_cap*P10</f>
         <v/>
       </c>
-      <c r="R10" s="34">
+      <c r="R10" s="36">
         <f>Q10*O10</f>
         <v/>
       </c>
-      <c r="S10" s="37">
+      <c r="S10" s="39">
         <f>E10*discount</f>
         <v/>
       </c>
-      <c r="T10" s="38">
+      <c r="T10" s="40">
         <f>S10*R10</f>
         <v/>
       </c>
-      <c r="U10" s="38">
+      <c r="U10" s="40">
         <f>(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,3,FALSE)</f>
         <v/>
       </c>
-      <c r="V10" s="38">
+      <c r="V10" s="40">
         <f>VLOOKUP(B10,country_opex,2,FALSE)*crew_factor</f>
         <v/>
       </c>
-      <c r="W10" s="38">
+      <c r="W10" s="40">
         <f>VLOOKUP(B10,country_opex,5,FALSE)</f>
         <v/>
       </c>
-      <c r="X10" s="38">
+      <c r="X10" s="40">
         <f>maint</f>
         <v/>
       </c>
-      <c r="Y10" s="38">
+      <c r="Y10" s="40">
         <f>VLOOKUP(B10,country_opex,7,FALSE)*ins_pct</f>
         <v/>
       </c>
-      <c r="Z10" s="38">
+      <c r="Z10" s="40">
         <f>charge_berth</f>
         <v/>
       </c>
-      <c r="AA10" s="38">
+      <c r="AA10" s="40">
         <f>U10+V10+W10+X10+Y10+Z10</f>
         <v/>
       </c>
-      <c r="AB10" s="38">
+      <c r="AB10" s="40">
         <f>VLOOKUP(B10,country_opex,7,FALSE)/dep_years</f>
         <v/>
       </c>
-      <c r="AC10" s="38">
+      <c r="AC10" s="40">
         <f>T10-AA10</f>
         <v/>
       </c>
-      <c r="AD10" s="35">
+      <c r="AD10" s="37">
         <f>IF(T10=0,"",AC10/T10)</f>
         <v/>
       </c>
-      <c r="AE10" s="36">
+      <c r="AE10" s="38">
         <f>IF(AC10&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/AC10)</f>
         <v/>
       </c>
-      <c r="AF10" s="33">
+      <c r="AF10" s="35">
         <f>((D10*O10/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D10*O10*VLOOKUP(B10,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG10" s="31" t="n">
+      <c r="AG10" s="33" t="n">
         <v>250000</v>
       </c>
-      <c r="AH10" s="32" t="inlineStr">
+      <c r="AH10" s="34" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="AI10" s="32" t="inlineStr">
+      <c r="AI10" s="34" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="AJ10" s="39" t="n">
+      <c r="AJ10" s="41" t="n">
         <v>0.9</v>
       </c>
-      <c r="AK10" s="34">
+      <c r="AK10" s="36">
         <f>IF(AG10="","",AG10*AJ10)</f>
         <v/>
       </c>
-      <c r="AL10" s="34">
+      <c r="AL10" s="36">
         <f>IF(OR(AG10="",R10=0),"",MIN(IF(AT10="",9.9E+99,AT10),FLOOR(AK10/R10,1)))</f>
         <v/>
       </c>
-      <c r="AM10" s="38">
-        <f>IF(AL10="","",AL10*T10)</f>
-        <v/>
-      </c>
-      <c r="AN10" s="36">
+      <c r="AM10" s="40">
+        <f>IF(AL10="","",AL10*IF(ABS(MOD(ABS((T10)),1)-0.5)&lt;1E-9,2*ROUND((T10)/2,0),ROUND((T10),0)))</f>
+        <v/>
+      </c>
+      <c r="AN10" s="38">
         <f>IF(OR(AG10="",R10=0),"",MIN(IF(AT10="",9.9E+99,AT10),AK10/R10))</f>
         <v/>
       </c>
-      <c r="AO10" s="38">
+      <c r="AO10" s="40">
         <f>IF(AN10="","",AN10*T10)</f>
         <v/>
       </c>
-      <c r="AP10" s="40" t="n"/>
-      <c r="AQ10" s="32" t="inlineStr">
+      <c r="AP10" s="42" t="n"/>
+      <c r="AQ10" s="34" t="inlineStr">
         <is>
           <t>Grounded</t>
         </is>
       </c>
-      <c r="AR10" s="41" t="n"/>
-      <c r="AS10" s="41" t="n"/>
-      <c r="AT10" s="42" t="n"/>
-      <c r="AU10" s="43">
-        <f>IF(((S10*pax_cap*load_thin*ROUND(K10*L10*revleg_thin,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_thin,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_thin*ROUND(K10*L10*revleg_thin,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_thin,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
-        <v/>
-      </c>
-      <c r="AV10" s="43">
-        <f>IF(((S10*pax_cap*load_mid*ROUND(K10*L10*revleg_mid,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_mid,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_mid*ROUND(K10*L10*revleg_mid,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_mid,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
-        <v/>
-      </c>
-      <c r="AW10" s="43">
-        <f>IF(((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
-        <v/>
-      </c>
-      <c r="AX10" s="44" t="inlineStr">
+      <c r="AR10" s="43" t="n"/>
+      <c r="AS10" s="43" t="n"/>
+      <c r="AT10" s="44" t="n"/>
+      <c r="AU10" s="45">
+        <f>IF(((S10*pax_cap*load_thin*IF(ABS(MOD(ABS((K10*L10*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_thin)/2,0),ROUND((K10*L10*revleg_thin),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_thin)/2,0),ROUND((K10*L10*revleg_thin),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_thin*IF(ABS(MOD(ABS((K10*L10*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_thin)/2,0),ROUND((K10*L10*revleg_thin),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_thin)/2,0),ROUND((K10*L10*revleg_thin),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AV10" s="45">
+        <f>IF(((S10*pax_cap*load_mid*IF(ABS(MOD(ABS((K10*L10*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_mid)/2,0),ROUND((K10*L10*revleg_mid),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_mid)/2,0),ROUND((K10*L10*revleg_mid),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_mid*IF(ABS(MOD(ABS((K10*L10*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_mid)/2,0),ROUND((K10*L10*revleg_mid),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_mid)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_mid)/2,0),ROUND((K10*L10*revleg_mid),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AW10" s="45">
+        <f>IF(((S10*pax_cap*load_full*IF(ABS(MOD(ABS((K10*L10*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_full)/2,0),ROUND((K10*L10*revleg_full),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_full)/2,0),ROUND((K10*L10*revleg_full),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*IF(ABS(MOD(ABS((K10*L10*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_full)/2,0),ROUND((K10*L10*revleg_full),0)))-(((battery/range_nm)*D10*IF(ABS(MOD(ABS((K10*L10*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((K10*L10*revleg_full)/2,0),ROUND((K10*L10*revleg_full),0))*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
+        <v/>
+      </c>
+      <c r="AX10" s="46" t="inlineStr">
         <is>
           <t>Sindalah is an ultra-premium yachting island (413-440 hotel rooms, 86-berth marina). NEOM inter-zone premium per-seat transfer modeled on Maldives/yacht-hub premium speedboat tier -&gt; $120.</t>
         </is>
       </c>
-      <c r="AY10" s="44" t="inlineStr">
+      <c r="AY10" s="46" t="inlineStr">
         <is>
           <t>NEOM Sindalah target: up to 2,400 guests/day by 2028 (NEOM official; Dezeen; Wikipedia) = ~876,000 guest-days/yr capacity; at ~3-4 night avg stay ~= ~250k arrivals/yr. Sindalah-&gt;Magna/Oxagon inter-zone transit is a SUBSET (R3) - recorded full Sindalah arrival proxy ~250k, low conf (not all transit to Magna/Oxagon).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="45" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>TOTAL / median</t>
         </is>
       </c>
-      <c r="T11" s="46">
+      <c r="T11" s="48">
         <f>SUM(T4:T10)</f>
         <v/>
       </c>
-      <c r="AC11" s="46">
+      <c r="AC11" s="48">
         <f>SUM(AC4:AC10)</f>
         <v/>
       </c>
-      <c r="AD11" s="47">
+      <c r="AD11" s="49">
         <f>IF(T11=0,"",AC11/T11)</f>
         <v/>
       </c>
-      <c r="AL11" s="48">
+      <c r="AL11" s="50">
         <f>SUM(AL4:AL10)</f>
         <v/>
       </c>
-      <c r="AM11" s="46">
+      <c r="AM11" s="48">
         <f>SUM(AM4:AM10)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>Fleet basis</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>Raw vessels (sum)</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t>Fleet (rounded once)</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="25" t="inlineStr">
         <is>
           <t>Market rev/yr (raw sum)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Saudi – Red Sea (Resort)</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>per_corridor_floor</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="49">
+      <c r="D15" s="51">
         <f>SUMIFS(AL4:AL10,A4:A10,"Saudi – Red Sea (Resort)",AP4:AP10,"=",AQ4:AQ10,"Grounded")</f>
         <v/>
       </c>
-      <c r="E15" s="50">
+      <c r="E15" s="52">
         <f>SUMIFS(AM4:AM10,A4:A10,"Saudi – Red Sea (Resort)",AP4:AP10,"=",AQ4:AQ10,"Grounded")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="45" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D16" s="48">
+      <c r="D16" s="50">
         <f>SUM(D15:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="46">
+      <c r="E16" s="48">
         <f>SUM(E15:E15)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>ESTIMATED DEMAND (country-median cascade; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="D17" s="51">
+      <c r="D17" s="53">
         <f>SUMIF(AQ4:AQ10,"Estimated",AL4:AL10)</f>
         <v/>
       </c>
-      <c r="E17" s="52">
+      <c r="E17" s="54">
         <f>SUMIF(AQ4:AQ10,"Estimated",AM4:AM10)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>FORWARD SAM (2030-dated; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="D18" s="51">
+      <c r="D18" s="53">
         <f>SUMIF(AQ4:AQ10,"Forward SAM",AL4:AL10)</f>
         <v/>
       </c>
-      <c r="E18" s="52">
+      <c r="E18" s="54">
         <f>SUMIF(AQ4:AQ10,"Forward SAM",AM4:AM10)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="53" t="inlineStr">
+      <c r="A20" s="55" t="inlineStr">
         <is>
           <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
         </is>
       </c>
-      <c r="C20" s="54" t="inlineStr">
+      <c r="C20" s="56" t="inlineStr">
         <is>
           <t>Shura Island hub → AMAALA (Triple Bay) (82.9nm)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="54" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>Jeddah → NEOM (Sindalah) (463.9nm)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="54" t="inlineStr">
+      <c r="C22" s="56" t="inlineStr">
         <is>
           <t>Jeddah gateway → The Red Sea archipelago (275.5nm)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="54" t="inlineStr">
+      <c r="C23" s="56" t="inlineStr">
         <is>
           <t>The Red Sea → NEOM (Sindalah) / Jeddah gateway (196.9nm)</t>
         </is>
@@ -3797,7 +3878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3814,401 +3895,402 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Market sizing — how the grounded floor builds into SOM → SAM → TAM</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Growth multipliers (bands: low / MID / high)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Multiplier</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Induced demand (k)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="20" t="n">
         <v>1.3</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="20" t="n">
         <v>1.8</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <v>2.5</v>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Faster/quieter product grows the crossing market beyond today's trips.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Mature capture rate (c)</t>
         </is>
       </c>
-      <c r="B6" s="39" t="n">
+      <c r="B6" s="41" t="n">
         <v>0.8934</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="C6" s="41" t="n">
         <v>0.8934</v>
       </c>
-      <c r="D6" s="39" t="n">
+      <c r="D6" s="41" t="n">
         <v>0.9434</v>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Navier's corridor share once it is the established premium default (vs 10% floor).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Journey GMV multiple (m)</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Whole island-journey wallet (transport+food+stay+experiences) as a multiple of the boat fare.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Greenfield network factor (g)</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>3.44</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="20" t="n">
         <v>4.9</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>6.36</v>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Width lever: addressable network vs the sourced subset (ID-based census).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Platform take rate</t>
         </is>
       </c>
-      <c r="C9" s="39" t="n">
+      <c r="C9" s="41" t="n">
         <v>0.18</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Super-app blended commission on journey GMV (derived line only).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>SOM capture rate (floor)</t>
         </is>
       </c>
-      <c r="C11" s="39" t="n">
-        <v>0.8934</v>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="C11" s="57">
+        <f>som_floor_rev/(ROUND(SUMPRODUCT(--('Corridor economics'!$AQ$4:$AQ$10="Grounded"),'Corridor economics'!$AG$4:$AG$10,'Corridor economics'!$E$4:$E$10),0))</f>
+        <v/>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Captive sole-operator capture (~89%) that builds the published floor; M_today = floor ÷ this = the true corridor spend pool.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>The ladder (live off the corridor floor)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Rung</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Definition</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>SOM floor — Navier transport rev/yr (PUBLISHED)</t>
         </is>
       </c>
-      <c r="C15" s="50">
+      <c r="C15" s="52">
         <f>som_floor_rev</f>
         <v/>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Live sum of grounded-floor corridor market-rev only (Floor bucket = Grounded; cascade-estimated rows held out). Matches growth.py _headline_anchor and deck TAM.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>M_today — full transport spend on sourced corridors</t>
-        </is>
-      </c>
-      <c r="C16" s="50">
-        <f>$C$15/$C$11</f>
-        <v/>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Anchor = SOM floor ÷ capture rate; recovers the whole crossing pool's premium-transfer spend today.</t>
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>M_today — model comparable-fare transport pool on sourced corridors</t>
+        </is>
+      </c>
+      <c r="C16" s="52">
+        <f>ROUND(SUMPRODUCT(--('Corridor economics'!$AQ$4:$AQ$10="Grounded"),'Corridor economics'!$AG$4:$AG$10,'Corridor economics'!$E$4:$E$10),0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Direct sum of sourced one-way demand × the disclosed model comparable fare on grounded corridors; includes any labelled premium re-fare applied above and is independent of display-rounded capture.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>SOM full network (~89% capture, today, +greenfield)</t>
         </is>
       </c>
-      <c r="B18" s="50">
+      <c r="B18" s="52">
         <f>$C$16*$C$11*$B$8</f>
         <v/>
       </c>
-      <c r="C18" s="50">
+      <c r="C18" s="52">
         <f>$C$16*$C$11*$C$8</f>
         <v/>
       </c>
-      <c r="D18" s="50">
+      <c r="D18" s="52">
         <f>$C$16*$C$11*$D$8</f>
         <v/>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>Floor posture (~89% captive capture, today's demand) extended across the whole mapped network.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>SAM — sourced corridors only (depth, no greenfield)</t>
         </is>
       </c>
-      <c r="B19" s="50">
+      <c r="B19" s="52">
         <f>$C$16*$B$5*$B$6</f>
         <v/>
       </c>
-      <c r="C19" s="50">
+      <c r="C19" s="52">
         <f>$C$16*$C$5*$C$6</f>
         <v/>
       </c>
-      <c r="D19" s="50">
+      <c r="D19" s="52">
         <f>$C$16*$D$5*$D$6</f>
         <v/>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Matured network on the sourced corridors alone: induced demand × mature capture.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>SAM — Navier transport rev @ full network (HEADLINE)</t>
         </is>
       </c>
-      <c r="B20" s="50">
+      <c r="B20" s="52">
         <f>$C$16*$B$5*$B$6*$B$8</f>
         <v/>
       </c>
-      <c r="C20" s="50">
+      <c r="C20" s="52">
         <f>$C$16*$C$5*$C$6*$C$8</f>
         <v/>
       </c>
-      <c r="D20" s="50">
+      <c r="D20" s="52">
         <f>$C$16*$D$5*$D$6*$D$8</f>
         <v/>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>Matured across the full addressable network: induced × mature capture × greenfield width.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Marine mobility TAM — induced marine-transfer market (LB-110)</t>
         </is>
       </c>
-      <c r="B21" s="50">
+      <c r="B21" s="52">
         <f>$C$16*$B$5*$B$8</f>
         <v/>
       </c>
-      <c r="C21" s="50">
+      <c r="C21" s="52">
         <f>$C$16*$C$5*$C$8</f>
         <v/>
       </c>
-      <c r="D21" s="50">
+      <c r="D21" s="52">
         <f>$C$16*$D$5*$D$8</f>
         <v/>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>SAM divided by leading-operator capture (= M_today × induced × greenfield). The full inducible water-transfer wallet at network maturity, before any capture constraint.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Journey GMV — induced crossing × multiple (was TAM journey GMV)</t>
         </is>
       </c>
-      <c r="B22" s="50">
+      <c r="B22" s="52">
         <f>$C$16*$B$5*$B$7*$B$8</f>
         <v/>
       </c>
-      <c r="C22" s="50">
+      <c r="C22" s="52">
         <f>$C$16*$C$5*$C$7*$C$8</f>
         <v/>
       </c>
-      <c r="D22" s="50">
+      <c r="D22" s="52">
         <f>$C$16*$D$5*$D$7*$D$8</f>
         <v/>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>Whole-journey spend (transport+food+stay+experiences) across the induced crossing market on the full network. Marine TAM × journey GMV multiple.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Journey GMV routed through Navier network</t>
         </is>
       </c>
-      <c r="B23" s="50">
+      <c r="B23" s="52">
         <f>$C$16*$B$5*$B$6*$B$7*$B$8</f>
         <v/>
       </c>
-      <c r="C23" s="50">
+      <c r="C23" s="52">
         <f>$C$16*$C$5*$C$6*$C$7*$C$8</f>
         <v/>
       </c>
-      <c r="D23" s="50">
+      <c r="D23" s="52">
         <f>$C$16*$D$5*$D$6*$D$7*$D$8</f>
         <v/>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>Journey GMV on Navier-carried trips only.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Partner platform revenue on Navier (LB-113 — on-Navier subset, not 18% of full Journey GMV)</t>
         </is>
       </c>
-      <c r="B24" s="50">
+      <c r="B24" s="52">
         <f>$C$16*$B$5*$B$6*$B$7*$B$8*$C$9</f>
         <v/>
       </c>
-      <c r="C24" s="50">
+      <c r="C24" s="52">
         <f>$C$16*$C$5*$C$6*$C$7*$C$8*$C$9</f>
         <v/>
       </c>
-      <c r="D24" s="50">
+      <c r="D24" s="52">
         <f>$C$16*$D$5*$D$6*$D$7*$D$8*$C$9</f>
         <v/>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>The super-app's own commission — the number a platform partner cares about.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="55" t="inlineStr">
+      <c r="A26" s="58" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B26" s="56" t="inlineStr">
+      <c r="B26" s="59" t="inlineStr">
         <is>
           <t>All rungs are one multiplication chain off M_today, which is live off the corridor floor. Change any input (a fare, a multiplier, the scenario) and the whole ladder moves. Bands (low/MID/high) are never single points; greenfield census is per-partner.</t>
         </is>

</xml_diff>